<commit_message>
20 morning update after delevery
</commit_message>
<xml_diff>
--- a/july 2026/Daily Reports/Final Execution SKU wise  july.xlsx
+++ b/july 2026/Daily Reports/Final Execution SKU wise  july.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\786\Desktop\Elite-Git\july 2026\Daily Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34033E70-8B84-42E3-B880-F6EBC8F85915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A20EE2B2-BB6B-4049-AA62-B7B36C3F47CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="887" activeTab="17" xr2:uid="{6D56E189-8B51-44FA-B14F-5373D35B2784}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="887" activeTab="20" xr2:uid="{6D56E189-8B51-44FA-B14F-5373D35B2784}"/>
   </bookViews>
   <sheets>
     <sheet name="last month" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1382" uniqueCount="40">
   <si>
     <t>Gate Pass</t>
   </si>
@@ -143,9 +143,6 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t>ok</t>
   </si>
   <si>
     <t>Executed</t>
@@ -661,7 +658,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
@@ -842,6 +839,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1523,12 +1526,12 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
@@ -1543,12 +1546,12 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1608,7 +1611,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -1620,7 +1623,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -1949,7 +1952,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>140</v>
@@ -2021,7 +2024,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>172</v>
@@ -2498,7 +2501,7 @@
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -2509,7 +2512,7 @@
       <c r="I2" s="62"/>
       <c r="L2" s="1"/>
       <c r="M2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N2" s="62"/>
       <c r="O2" s="62"/>
@@ -2677,7 +2680,7 @@
         <v>12</v>
       </c>
       <c r="V7" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="W7" s="59" t="s">
         <v>26</v>
@@ -2783,7 +2786,7 @@
     <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12">
@@ -2827,7 +2830,7 @@
     <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>210</v>
@@ -3277,7 +3280,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -3288,7 +3291,7 @@
       <c r="I2" s="62"/>
       <c r="L2" s="1"/>
       <c r="M2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N2" s="62"/>
       <c r="O2" s="62"/>
@@ -3571,7 +3574,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>100</v>
@@ -3639,7 +3642,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>192</v>
@@ -3739,7 +3742,7 @@
     <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13" s="11"/>
       <c r="B13" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="12"/>
@@ -4146,7 +4149,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -4158,7 +4161,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -4434,7 +4437,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -4478,7 +4481,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -4944,7 +4947,7 @@
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -4955,7 +4958,7 @@
       <c r="I2" s="62"/>
       <c r="L2" s="1"/>
       <c r="M2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N2" s="62"/>
       <c r="O2" s="62"/>
@@ -5194,7 +5197,7 @@
     <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>155</v>
@@ -5257,7 +5260,7 @@
     <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>172</v>
@@ -5332,7 +5335,7 @@
     <row r="12" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A12" s="11"/>
       <c r="B12" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12">
@@ -5789,7 +5792,7 @@
     <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -5800,7 +5803,7 @@
       <c r="I2" s="62"/>
       <c r="L2" s="1"/>
       <c r="M2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N2" s="62"/>
       <c r="O2" s="62"/>
@@ -6099,7 +6102,7 @@
     <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>90</v>
@@ -6162,7 +6165,7 @@
     <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>308</v>
@@ -6244,7 +6247,7 @@
       </c>
       <c r="L12" s="11"/>
       <c r="M12" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N12" s="12"/>
       <c r="O12" s="12">
@@ -6610,7 +6613,7 @@
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -6621,7 +6624,7 @@
       <c r="I2" s="62"/>
       <c r="L2" s="1"/>
       <c r="M2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N2" s="62"/>
       <c r="O2" s="62"/>
@@ -6938,7 +6941,7 @@
     <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>242</v>
@@ -7004,7 +7007,7 @@
     <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>72</v>
@@ -7072,7 +7075,7 @@
     <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="11"/>
       <c r="B12" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12">
@@ -7492,7 +7495,7 @@
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -7503,7 +7506,7 @@
       <c r="I2" s="62"/>
       <c r="L2" s="1"/>
       <c r="M2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N2" s="62"/>
       <c r="O2" s="62"/>
@@ -7816,7 +7819,7 @@
     <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>150</v>
@@ -7884,7 +7887,7 @@
     <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -8309,7 +8312,7 @@
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -8320,7 +8323,7 @@
       <c r="I2" s="62"/>
       <c r="L2" s="1"/>
       <c r="M2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N2" s="62"/>
       <c r="O2" s="62"/>
@@ -8635,7 +8638,7 @@
     <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>222</v>
@@ -8701,7 +8704,7 @@
     <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>460</v>
@@ -8769,7 +8772,7 @@
     <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="11"/>
       <c r="B12" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C12" s="12"/>
       <c r="D12" s="12">
@@ -9180,7 +9183,7 @@
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -9191,7 +9194,7 @@
       <c r="I2" s="62"/>
       <c r="L2" s="1"/>
       <c r="M2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N2" s="62"/>
       <c r="O2" s="62"/>
@@ -9338,7 +9341,7 @@
       <c r="M7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="N7" s="58" t="s">
+      <c r="N7" s="75" t="s">
         <v>6</v>
       </c>
       <c r="O7" s="56" t="s">
@@ -9347,8 +9350,8 @@
       <c r="P7" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="Q7" s="45" t="s">
-        <v>8</v>
+      <c r="Q7" s="56" t="s">
+        <v>12</v>
       </c>
       <c r="R7" s="45" t="s">
         <v>13</v>
@@ -9356,11 +9359,11 @@
       <c r="S7" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="T7" s="12" t="s">
+      <c r="T7" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="U7" s="12" t="s">
-        <v>8</v>
+      <c r="U7" s="45" t="s">
+        <v>12</v>
       </c>
       <c r="V7" s="12" t="s">
         <v>27</v>
@@ -9407,23 +9410,34 @@
         <f>B8</f>
         <v>Furqan</v>
       </c>
-      <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-      <c r="P8" s="12"/>
+      <c r="N8" s="12">
+        <v>76</v>
+      </c>
+      <c r="O8" s="12">
+        <v>26</v>
+      </c>
+      <c r="P8" s="12">
+        <v>20</v>
+      </c>
       <c r="Q8" s="28">
-        <f t="shared" ref="Q8:Q13" si="0">SUM(O8:P8)/20</f>
-        <v>0</v>
-      </c>
-      <c r="R8" s="12"/>
-      <c r="S8" s="12"/>
+        <v>0</v>
+      </c>
+      <c r="R8" s="12">
+        <v>26</v>
+      </c>
+      <c r="S8" s="12">
+        <v>0</v>
+      </c>
       <c r="T8" s="12"/>
       <c r="U8" s="28">
-        <f>SUM(R8:T8)/20</f>
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="V8">
-        <f>SUM(N8:P8,R8,S8,T8)/40</f>
-        <v>0</v>
+        <f>SUM(N8:U8)/40</f>
+        <v>4.3499999999999996</v>
+      </c>
+      <c r="W8" s="76">
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.35">
@@ -9453,7 +9467,7 @@
         <v>95</v>
       </c>
       <c r="J9" s="44">
-        <f t="shared" ref="J9:J12" si="1">SUM(C9:I9)/40</f>
+        <f t="shared" ref="J9:J12" si="0">SUM(C9:I9)/40</f>
         <v>10.25</v>
       </c>
       <c r="K9" s="44">
@@ -9464,29 +9478,40 @@
         <f>B9</f>
         <v>Salman</v>
       </c>
-      <c r="N9" s="12"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="12"/>
+      <c r="N9" s="12">
+        <v>155</v>
+      </c>
+      <c r="O9" s="12">
+        <v>20</v>
+      </c>
+      <c r="P9" s="12">
+        <v>30</v>
+      </c>
       <c r="Q9" s="28">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="R9" s="12"/>
-      <c r="S9" s="12"/>
+        <v>0</v>
+      </c>
+      <c r="R9" s="12">
+        <v>65</v>
+      </c>
+      <c r="S9" s="12">
+        <v>0</v>
+      </c>
       <c r="T9" s="12"/>
       <c r="U9" s="28">
-        <f t="shared" ref="U9:U13" si="2">SUM(R9:T9)/20</f>
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="V9">
-        <f>SUM(N9:P9,R9,S9,T9)/40</f>
-        <v>0</v>
+        <f t="shared" ref="V9:V12" si="1">SUM(N9:U9)/40</f>
+        <v>8.75</v>
+      </c>
+      <c r="W9" s="76">
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>74</v>
@@ -9510,7 +9535,7 @@
         <v>110</v>
       </c>
       <c r="J10" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>17.850000000000001</v>
       </c>
       <c r="K10" s="44">
@@ -9521,29 +9546,40 @@
         <f>B10</f>
         <v>Zesahn</v>
       </c>
-      <c r="N10" s="12"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="12"/>
+      <c r="N10" s="12">
+        <v>74</v>
+      </c>
+      <c r="O10" s="12">
+        <v>30</v>
+      </c>
+      <c r="P10" s="12">
+        <v>30</v>
+      </c>
       <c r="Q10" s="28">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="R10" s="12"/>
-      <c r="S10" s="12"/>
+        <v>0</v>
+      </c>
+      <c r="R10" s="12">
+        <v>470</v>
+      </c>
+      <c r="S10" s="12">
+        <v>0</v>
+      </c>
       <c r="T10" s="12"/>
       <c r="U10" s="28">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="V10">
-        <f>SUM(N10:P10,R10,S10,T10)/40</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>17.850000000000001</v>
+      </c>
+      <c r="W10" s="76">
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>180</v>
@@ -9567,7 +9603,7 @@
         <v>50</v>
       </c>
       <c r="J11" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="K11" s="44">
@@ -9578,23 +9614,34 @@
         <f>B11</f>
         <v>Umair</v>
       </c>
-      <c r="N11" s="12"/>
-      <c r="O11" s="12"/>
-      <c r="P11" s="12"/>
+      <c r="N11" s="12">
+        <v>60</v>
+      </c>
+      <c r="O11" s="12">
+        <v>20</v>
+      </c>
+      <c r="P11" s="12">
+        <v>20</v>
+      </c>
       <c r="Q11" s="28">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="R11" s="12"/>
-      <c r="S11" s="12"/>
+        <v>0</v>
+      </c>
+      <c r="R11" s="12">
+        <v>30</v>
+      </c>
+      <c r="S11" s="12">
+        <v>0</v>
+      </c>
       <c r="T11" s="12"/>
       <c r="U11" s="28">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="V11">
-        <f>SUM(N11:P11,R11,S11,T11)/40</f>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="W11" s="76">
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.35">
@@ -9610,7 +9657,7 @@
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
       <c r="J12" s="44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L12" s="11"/>
@@ -9621,19 +9668,13 @@
       <c r="N12" s="12"/>
       <c r="O12" s="12"/>
       <c r="P12" s="12"/>
-      <c r="Q12" s="28">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="Q12" s="28"/>
       <c r="R12" s="12"/>
       <c r="S12" s="12"/>
       <c r="T12" s="12"/>
-      <c r="U12" s="28">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="U12" s="28"/>
       <c r="V12">
-        <f>SUM(N12:P12,R12,S12,T12)/40</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
@@ -9653,47 +9694,41 @@
       <c r="N13" s="12"/>
       <c r="O13" s="12"/>
       <c r="P13" s="12"/>
-      <c r="Q13" s="28">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="Q13" s="28"/>
       <c r="R13" s="12"/>
       <c r="S13" s="12"/>
       <c r="T13" s="12"/>
-      <c r="U13" s="28">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
+      <c r="U13" s="28"/>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="13"/>
       <c r="B14" s="10"/>
       <c r="C14" s="14">
-        <f t="shared" ref="C14:I14" si="3">SUM(C8:C13)</f>
+        <f t="shared" ref="C14:I14" si="2">SUM(C8:C13)</f>
         <v>485</v>
       </c>
       <c r="D14" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>136</v>
       </c>
       <c r="E14" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>180</v>
       </c>
       <c r="F14" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G14" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>668</v>
       </c>
       <c r="H14" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I14" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>281</v>
       </c>
       <c r="J14" s="35">
@@ -9703,36 +9738,36 @@
       <c r="L14" s="13"/>
       <c r="M14" s="10"/>
       <c r="N14" s="14">
-        <f t="shared" ref="N14:U14" si="4">SUM(N8:N13)</f>
-        <v>0</v>
+        <f t="shared" ref="N14:U14" si="3">SUM(N8:N13)</f>
+        <v>365</v>
       </c>
       <c r="O14" s="14">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>96</v>
       </c>
       <c r="P14" s="14">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>100</v>
       </c>
       <c r="Q14" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="R14" s="14">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>591</v>
       </c>
       <c r="S14" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="T14" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="U14" s="14">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>246</v>
       </c>
       <c r="V14" s="35" t="e">
         <f>N14+O14+P14+#REF!+R14+S14+T14</f>
@@ -9750,23 +9785,23 @@
         <v>6.8</v>
       </c>
       <c r="E15" s="13">
-        <f t="shared" ref="E15:I15" si="5">E14/20</f>
+        <f t="shared" ref="E15:I15" si="4">E14/20</f>
         <v>9</v>
       </c>
       <c r="F15" s="13">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="G15" s="13">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>33.4</v>
       </c>
       <c r="H15" s="13">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="I15" s="13">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>14.05</v>
       </c>
       <c r="K15" t="s">
@@ -9779,23 +9814,23 @@
       <c r="N15" s="13"/>
       <c r="O15" s="13">
         <f>O14/20</f>
-        <v>0</v>
+        <v>4.8</v>
       </c>
       <c r="P15" s="13">
-        <f t="shared" ref="P15" si="6">P14/20</f>
-        <v>0</v>
+        <f t="shared" ref="P15" si="5">P14/20</f>
+        <v>5</v>
       </c>
       <c r="Q15" s="13"/>
       <c r="R15" s="13">
-        <f t="shared" ref="R15:T15" si="7">R14/20</f>
-        <v>0</v>
+        <f t="shared" ref="R15:T15" si="6">R14/20</f>
+        <v>29.55</v>
       </c>
       <c r="S15" s="13">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="T15" s="13">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="U15" s="13"/>
@@ -9810,27 +9845,27 @@
         <v>485</v>
       </c>
       <c r="D16" s="36">
-        <f t="shared" ref="D16:I16" si="8">D15+D14</f>
+        <f t="shared" ref="D16:I16" si="7">D15+D14</f>
         <v>142.80000000000001</v>
       </c>
       <c r="E16" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>189</v>
       </c>
       <c r="F16" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="G16" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>701.4</v>
       </c>
       <c r="H16" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="I16" s="36">
-        <f t="shared" si="8"/>
+        <f t="shared" si="7"/>
         <v>295.05</v>
       </c>
       <c r="L16" s="13"/>
@@ -9839,27 +9874,27 @@
       </c>
       <c r="N16" s="36">
         <f>N15+N14</f>
-        <v>0</v>
+        <v>365</v>
       </c>
       <c r="O16" s="36">
-        <f t="shared" ref="O16:P16" si="9">O15+O14</f>
-        <v>0</v>
+        <f t="shared" ref="O16:P16" si="8">O15+O14</f>
+        <v>100.8</v>
       </c>
       <c r="P16" s="36">
-        <f t="shared" si="9"/>
-        <v>0</v>
+        <f t="shared" si="8"/>
+        <v>105</v>
       </c>
       <c r="Q16" s="36"/>
       <c r="R16" s="36">
-        <f t="shared" ref="R16:T16" si="10">R15+R14</f>
-        <v>0</v>
+        <f t="shared" ref="R16:T16" si="9">R15+R14</f>
+        <v>620.54999999999995</v>
       </c>
       <c r="S16" s="36">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="T16" s="36">
-        <f t="shared" si="10"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="U16" s="36"/>
@@ -9874,27 +9909,27 @@
         <v>12.125</v>
       </c>
       <c r="D17" s="36">
-        <f t="shared" ref="D17:I17" si="11">D14/40</f>
+        <f t="shared" ref="D17:I17" si="10">D14/40</f>
         <v>3.4</v>
       </c>
       <c r="E17" s="36">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>4.5</v>
       </c>
       <c r="F17" s="36">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="G17" s="36">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>16.7</v>
       </c>
       <c r="H17" s="36">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="I17" s="36">
-        <f t="shared" si="11"/>
+        <f t="shared" si="10"/>
         <v>7.0250000000000004</v>
       </c>
       <c r="J17" s="35">
@@ -9907,33 +9942,33 @@
       </c>
       <c r="N17" s="36">
         <f>N14/40</f>
-        <v>0</v>
+        <v>9.125</v>
       </c>
       <c r="O17" s="36">
-        <f t="shared" ref="O17:P17" si="12">O14/40</f>
-        <v>0</v>
+        <f t="shared" ref="O17:P17" si="11">O14/40</f>
+        <v>2.4</v>
       </c>
       <c r="P17" s="36">
-        <f t="shared" si="12"/>
-        <v>0</v>
+        <f t="shared" si="11"/>
+        <v>2.5</v>
       </c>
       <c r="Q17" s="36"/>
       <c r="R17" s="36">
-        <f t="shared" ref="R17:T17" si="13">R14/40</f>
-        <v>0</v>
+        <f t="shared" ref="R17:T17" si="12">R14/40</f>
+        <v>14.775</v>
       </c>
       <c r="S17" s="36">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="T17" s="36">
-        <f t="shared" si="13"/>
+        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="U17" s="36"/>
       <c r="V17" s="35">
         <f>SUM(N17:T17)</f>
-        <v>0</v>
+        <v>28.8</v>
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.35">
@@ -10018,7 +10053,7 @@
     <row r="2" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -10031,7 +10066,7 @@
       <c r="K2" s="63"/>
       <c r="N2" s="1"/>
       <c r="O2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P2" s="62"/>
       <c r="Q2" s="62"/>
@@ -10043,7 +10078,7 @@
       <c r="W2" s="62"/>
       <c r="X2" s="63"/>
       <c r="AB2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.35">
@@ -10290,7 +10325,7 @@
         <v>46174</v>
       </c>
       <c r="O8" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P8" s="12">
         <v>284</v>
@@ -10456,7 +10491,7 @@
       </c>
       <c r="N10" s="27"/>
       <c r="O10" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="P10" s="12">
         <v>86</v>
@@ -10574,7 +10609,7 @@
     <row r="12" spans="1:30" x14ac:dyDescent="0.35">
       <c r="A12" s="11"/>
       <c r="B12" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" s="12">
         <v>382</v>
@@ -11055,7 +11090,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -11067,7 +11102,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -11257,13 +11292,13 @@
       <c r="B8" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
-      <c r="I8" s="12"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="29"/>
       <c r="J8" s="28">
         <f>SUM(G8:I8)/20</f>
         <v>0</v>
@@ -11273,22 +11308,22 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M8" s="27"/>
       <c r="N8" s="10" t="str">
         <f>B8</f>
         <v>Furqan</v>
       </c>
-      <c r="O8" s="12"/>
-      <c r="P8" s="12"/>
-      <c r="Q8" s="12"/>
-      <c r="R8" s="28">
+      <c r="O8" s="29"/>
+      <c r="P8" s="29"/>
+      <c r="Q8" s="29"/>
+      <c r="R8" s="29">
         <f t="shared" ref="R8:R13" si="0">SUM(P8:Q8)/20</f>
         <v>0</v>
       </c>
-      <c r="S8" s="12"/>
-      <c r="T8" s="12"/>
+      <c r="S8" s="29"/>
+      <c r="T8" s="29"/>
       <c r="U8" s="12"/>
       <c r="V8" s="28">
         <f>SUM(S8:U8)/20</f>
@@ -11304,13 +11339,13 @@
       <c r="B9" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="29"/>
       <c r="J9" s="28">
         <f t="shared" ref="J9:J13" si="1">SUM(G9:I9)/20</f>
         <v>0</v>
@@ -11320,22 +11355,22 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M9" s="27"/>
       <c r="N9" s="10" t="str">
         <f>B9</f>
         <v>Salman</v>
       </c>
-      <c r="O9" s="12"/>
-      <c r="P9" s="12"/>
-      <c r="Q9" s="12"/>
-      <c r="R9" s="28">
+      <c r="O9" s="29"/>
+      <c r="P9" s="29"/>
+      <c r="Q9" s="29"/>
+      <c r="R9" s="29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="S9" s="12"/>
-      <c r="T9" s="12"/>
+      <c r="S9" s="29"/>
+      <c r="T9" s="29"/>
       <c r="U9" s="12"/>
       <c r="V9" s="28">
         <f t="shared" ref="V9:V13" si="2">SUM(S9:U9)/20</f>
@@ -11349,15 +11384,15 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
+        <v>37</v>
+      </c>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="29"/>
       <c r="J10" s="28">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -11367,22 +11402,22 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="M10" s="27"/>
       <c r="N10" s="10" t="str">
         <f>B10</f>
         <v>Zesahn</v>
       </c>
-      <c r="O10" s="12"/>
-      <c r="P10" s="12"/>
-      <c r="Q10" s="12"/>
-      <c r="R10" s="28">
+      <c r="O10" s="29"/>
+      <c r="P10" s="29"/>
+      <c r="Q10" s="29"/>
+      <c r="R10" s="29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="S10" s="12"/>
-      <c r="T10" s="12"/>
+      <c r="S10" s="29"/>
+      <c r="T10" s="29"/>
       <c r="U10" s="12"/>
       <c r="V10" s="28">
         <f t="shared" si="2"/>
@@ -11396,15 +11431,15 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
+        <v>31</v>
+      </c>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
+      <c r="I11" s="29"/>
       <c r="J11" s="28">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -11418,15 +11453,15 @@
         <f>B11</f>
         <v>Umair</v>
       </c>
-      <c r="O11" s="12"/>
-      <c r="P11" s="12"/>
-      <c r="Q11" s="12"/>
-      <c r="R11" s="28">
+      <c r="O11" s="29"/>
+      <c r="P11" s="29"/>
+      <c r="Q11" s="29"/>
+      <c r="R11" s="29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="S11" s="12"/>
-      <c r="T11" s="12"/>
+      <c r="S11" s="29"/>
+      <c r="T11" s="29"/>
       <c r="U11" s="12"/>
       <c r="V11" s="28">
         <f t="shared" si="2"/>
@@ -11442,13 +11477,13 @@
       <c r="B12" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="29"/>
+      <c r="I12" s="29"/>
       <c r="J12" s="28">
         <f t="shared" si="1"/>
         <v>0</v>
@@ -11462,15 +11497,15 @@
         <f>B12</f>
         <v>Mubeen</v>
       </c>
-      <c r="O12" s="12"/>
-      <c r="P12" s="12"/>
-      <c r="Q12" s="12"/>
-      <c r="R12" s="28">
+      <c r="O12" s="29"/>
+      <c r="P12" s="29"/>
+      <c r="Q12" s="29"/>
+      <c r="R12" s="29">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="S12" s="12"/>
-      <c r="T12" s="12"/>
+      <c r="S12" s="29"/>
+      <c r="T12" s="29"/>
       <c r="U12" s="12"/>
       <c r="V12" s="28">
         <f t="shared" si="2"/>
@@ -11817,7 +11852,7 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C45487-B908-4B5C-9BA4-6B5B2A14CAC7}">
-  <dimension ref="A1:X19"/>
+  <dimension ref="A1:W19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3.90625" bestFit="1" customWidth="1"/>
@@ -11828,16 +11863,15 @@
     <col min="6" max="6" width="3.08984375" bestFit="1" customWidth="1"/>
     <col min="7" max="8" width="4.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="3.54296875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="3.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.453125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="4.26953125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="0" hidden="1" customWidth="1"/>
+    <col min="12" max="12" width="3.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="4.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -11847,7 +11881,7 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="L1" s="1"/>
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
       <c r="O1" s="1"/>
@@ -11857,12 +11891,11 @@
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
-    </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -11871,21 +11904,20 @@
       <c r="G2" s="62"/>
       <c r="H2" s="62"/>
       <c r="I2" s="62"/>
-      <c r="J2" s="63"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="61" t="s">
-        <v>36</v>
-      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="61" t="s">
+        <v>35</v>
+      </c>
+      <c r="N2" s="62"/>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
       <c r="Q2" s="62"/>
       <c r="R2" s="62"/>
       <c r="S2" s="62"/>
       <c r="T2" s="62"/>
-      <c r="U2" s="62"/>
-      <c r="V2" s="63"/>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="U2" s="63"/>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="64"/>
       <c r="C3" s="65"/>
@@ -11895,19 +11927,18 @@
       <c r="G3" s="65"/>
       <c r="H3" s="65"/>
       <c r="I3" s="65"/>
-      <c r="J3" s="66"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="64"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="64"/>
+      <c r="N3" s="65"/>
       <c r="O3" s="65"/>
       <c r="P3" s="65"/>
       <c r="Q3" s="65"/>
       <c r="R3" s="65"/>
       <c r="S3" s="65"/>
       <c r="T3" s="65"/>
-      <c r="U3" s="65"/>
-      <c r="V3" s="66"/>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="U3" s="66"/>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="B4" s="64"/>
       <c r="C4" s="65"/>
@@ -11917,19 +11948,18 @@
       <c r="G4" s="65"/>
       <c r="H4" s="65"/>
       <c r="I4" s="65"/>
-      <c r="J4" s="66"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="64"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="64"/>
+      <c r="N4" s="65"/>
       <c r="O4" s="65"/>
       <c r="P4" s="65"/>
       <c r="Q4" s="65"/>
       <c r="R4" s="65"/>
       <c r="S4" s="65"/>
       <c r="T4" s="65"/>
-      <c r="U4" s="65"/>
-      <c r="V4" s="66"/>
-    </row>
-    <row r="5" spans="1:24" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="U4" s="66"/>
+    </row>
+    <row r="5" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="1"/>
       <c r="B5" s="67"/>
       <c r="C5" s="68"/>
@@ -11939,19 +11969,18 @@
       <c r="G5" s="68"/>
       <c r="H5" s="68"/>
       <c r="I5" s="68"/>
-      <c r="J5" s="69"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="67"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="67"/>
+      <c r="N5" s="68"/>
       <c r="O5" s="68"/>
       <c r="P5" s="68"/>
       <c r="Q5" s="68"/>
       <c r="R5" s="68"/>
       <c r="S5" s="68"/>
       <c r="T5" s="68"/>
-      <c r="U5" s="68"/>
-      <c r="V5" s="69"/>
-    </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="U5" s="69"/>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
       <c r="B6" s="2"/>
       <c r="C6" s="3" t="s">
@@ -11967,25 +11996,24 @@
       </c>
       <c r="H6" s="71"/>
       <c r="I6" s="71"/>
-      <c r="J6" s="72"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="3" t="s">
+      <c r="L6" s="1"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="P6" s="70" t="s">
+      <c r="O6" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="Q6" s="71"/>
-      <c r="R6" s="72"/>
-      <c r="S6" s="71" t="s">
+      <c r="P6" s="71"/>
+      <c r="Q6" s="72"/>
+      <c r="R6" s="71" t="s">
         <v>3</v>
       </c>
+      <c r="S6" s="71"/>
       <c r="T6" s="71"/>
-      <c r="U6" s="71"/>
-      <c r="V6" s="72"/>
-    </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="U6" s="72"/>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>4</v>
       </c>
@@ -12014,52 +12042,49 @@
         <v>12</v>
       </c>
       <c r="J7" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="L7" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="M7" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="N7" s="75" t="s">
+        <v>6</v>
+      </c>
+      <c r="O7" s="56" t="s">
+        <v>13</v>
+      </c>
+      <c r="P7" s="56" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q7" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="K7" s="12" t="s">
+      <c r="R7" s="45" t="s">
+        <v>13</v>
+      </c>
+      <c r="S7" s="45" t="s">
+        <v>7</v>
+      </c>
+      <c r="T7" s="45" t="s">
+        <v>12</v>
+      </c>
+      <c r="U7" s="45" t="s">
+        <v>8</v>
+      </c>
+      <c r="V7" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="L7" s="12" t="s">
+      <c r="W7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="M7" s="10" t="s">
-        <v>4</v>
-      </c>
-      <c r="N7" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="O7" s="58" t="s">
-        <v>6</v>
-      </c>
-      <c r="P7" s="56" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q7" s="56" t="s">
-        <v>11</v>
-      </c>
-      <c r="R7" s="45" t="s">
-        <v>8</v>
-      </c>
-      <c r="S7" s="45" t="s">
-        <v>13</v>
-      </c>
-      <c r="T7" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="U7" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="V7" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="W7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="X7" s="12" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A8" s="27"/>
       <c r="B8" s="10" t="s">
         <v>17</v>
@@ -12071,183 +12096,183 @@
       <c r="G8" s="12"/>
       <c r="H8" s="12"/>
       <c r="I8" s="12"/>
-      <c r="J8" s="28">
-        <f>SUM(G8:I8)/20</f>
-        <v>0</v>
-      </c>
-      <c r="K8">
-        <f t="shared" ref="K8:K13" si="0">SUM(C8:F8,G8,H8,I8)/40</f>
-        <v>0</v>
-      </c>
-      <c r="L8" s="44" t="s">
-        <v>29</v>
-      </c>
-      <c r="M8" s="27"/>
-      <c r="N8" s="10" t="str">
+      <c r="J8">
+        <f>SUM(C8:F8,G8,H8,I8)/40</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="44"/>
+      <c r="L8" s="27"/>
+      <c r="M8" s="10" t="str">
         <f>B8</f>
         <v>Furqan</v>
       </c>
+      <c r="N8" s="12"/>
       <c r="O8" s="12"/>
       <c r="P8" s="12"/>
-      <c r="Q8" s="12"/>
-      <c r="R8" s="28">
-        <f t="shared" ref="R8:R13" si="1">SUM(P8:Q8)/20</f>
-        <v>0</v>
-      </c>
+      <c r="Q8" s="28"/>
+      <c r="R8" s="12"/>
       <c r="S8" s="12"/>
       <c r="T8" s="12"/>
-      <c r="U8" s="12"/>
-      <c r="V8" s="28">
-        <f>SUM(S8:U8)/20</f>
-        <v>0</v>
-      </c>
-      <c r="W8">
-        <f t="shared" ref="W8:W13" si="2">SUM(O8:Q8,S8,T8,U8)/40</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="U8" s="28"/>
+      <c r="V8">
+        <f t="shared" ref="V8:V13" si="0">SUM(N8:P8,R8,S8,T8)/40</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A9" s="27"/>
       <c r="B9" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="28">
-        <f t="shared" ref="J9:J13" si="3">SUM(G9:I9)/20</f>
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="L9" s="44" t="s">
-        <v>29</v>
-      </c>
-      <c r="M9" s="27"/>
-      <c r="N9" s="10" t="str">
+      <c r="C9" s="12">
+        <v>132</v>
+      </c>
+      <c r="D9" s="12">
+        <v>12</v>
+      </c>
+      <c r="E9" s="12">
+        <v>12</v>
+      </c>
+      <c r="F9" s="12">
+        <v>0</v>
+      </c>
+      <c r="G9" s="12">
+        <v>77</v>
+      </c>
+      <c r="H9" s="12">
+        <v>30</v>
+      </c>
+      <c r="I9" s="12">
+        <v>77</v>
+      </c>
+      <c r="J9">
+        <f>SUM(C9:F9,G9,H9,I9)/40</f>
+        <v>8.5</v>
+      </c>
+      <c r="K9" s="44">
+        <v>7</v>
+      </c>
+      <c r="L9" s="27"/>
+      <c r="M9" s="10" t="str">
         <f>B9</f>
         <v>Salman</v>
       </c>
+      <c r="N9" s="12"/>
       <c r="O9" s="12"/>
       <c r="P9" s="12"/>
-      <c r="Q9" s="12"/>
-      <c r="R9" s="28">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="Q9" s="28"/>
+      <c r="R9" s="12"/>
       <c r="S9" s="12"/>
       <c r="T9" s="12"/>
-      <c r="U9" s="12"/>
-      <c r="V9" s="28">
-        <f t="shared" ref="V9:V13" si="4">SUM(S9:U9)/20</f>
-        <v>0</v>
-      </c>
-      <c r="W9">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="U9" s="28"/>
+      <c r="V9">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="28">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="L10" s="44" t="s">
-        <v>29</v>
-      </c>
-      <c r="M10" s="27"/>
-      <c r="N10" s="10" t="str">
+        <v>37</v>
+      </c>
+      <c r="C10" s="12">
+        <v>202</v>
+      </c>
+      <c r="D10" s="12">
+        <v>66</v>
+      </c>
+      <c r="E10" s="12">
+        <v>66</v>
+      </c>
+      <c r="F10" s="12">
+        <v>0</v>
+      </c>
+      <c r="G10" s="12">
+        <v>126</v>
+      </c>
+      <c r="H10" s="12">
+        <v>126</v>
+      </c>
+      <c r="I10" s="12">
+        <v>212</v>
+      </c>
+      <c r="J10">
+        <f>SUM(C10:F10,G10,H10,I10)/40</f>
+        <v>19.95</v>
+      </c>
+      <c r="K10" s="44">
+        <v>16</v>
+      </c>
+      <c r="L10" s="27"/>
+      <c r="M10" s="10" t="str">
         <f>B10</f>
         <v>Zesahn</v>
       </c>
+      <c r="N10" s="12"/>
       <c r="O10" s="12"/>
       <c r="P10" s="12"/>
-      <c r="Q10" s="12"/>
-      <c r="R10" s="28">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="Q10" s="28"/>
+      <c r="R10" s="12"/>
       <c r="S10" s="12"/>
       <c r="T10" s="12"/>
-      <c r="U10" s="12"/>
-      <c r="V10" s="28">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="W10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="U10" s="28"/>
+      <c r="V10">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="28">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K11">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="L11" s="41" t="s">
-        <v>29</v>
-      </c>
-      <c r="M11" s="11"/>
-      <c r="N11" s="10" t="str">
+        <v>31</v>
+      </c>
+      <c r="C11" s="12">
+        <v>420</v>
+      </c>
+      <c r="D11" s="12">
+        <v>86</v>
+      </c>
+      <c r="E11" s="12">
+        <v>86</v>
+      </c>
+      <c r="F11" s="12">
+        <v>0</v>
+      </c>
+      <c r="G11" s="12">
+        <v>160</v>
+      </c>
+      <c r="H11" s="12">
+        <v>80</v>
+      </c>
+      <c r="I11" s="12">
+        <v>80</v>
+      </c>
+      <c r="J11">
+        <f>SUM(C11:F11,G11,H11,I11)/40</f>
+        <v>22.8</v>
+      </c>
+      <c r="K11" s="41">
+        <v>10</v>
+      </c>
+      <c r="L11" s="11"/>
+      <c r="M11" s="10" t="str">
         <f>B11</f>
         <v>Umair</v>
       </c>
+      <c r="N11" s="12"/>
       <c r="O11" s="12"/>
       <c r="P11" s="12"/>
-      <c r="Q11" s="12"/>
-      <c r="R11" s="28">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="Q11" s="28"/>
+      <c r="R11" s="12"/>
       <c r="S11" s="12"/>
       <c r="T11" s="12"/>
-      <c r="U11" s="12"/>
-      <c r="V11" s="28">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="W11">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="U11" s="28"/>
+      <c r="V11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="11"/>
       <c r="B12" s="11" t="s">
         <v>19</v>
@@ -12259,42 +12284,30 @@
       <c r="G12" s="12"/>
       <c r="H12" s="12"/>
       <c r="I12" s="12"/>
-      <c r="J12" s="28">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="L12" s="41" t="s">
-        <v>29</v>
-      </c>
-      <c r="M12" s="11"/>
-      <c r="N12" s="10" t="str">
+      <c r="J12">
+        <f>SUM(C12:F12,G12,H12,I12)/40</f>
+        <v>0</v>
+      </c>
+      <c r="K12" s="41"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="10" t="str">
         <f>B12</f>
         <v>Mubeen</v>
       </c>
+      <c r="N12" s="12"/>
       <c r="O12" s="12"/>
       <c r="P12" s="12"/>
-      <c r="Q12" s="12"/>
-      <c r="R12" s="28">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="Q12" s="28"/>
+      <c r="R12" s="12"/>
       <c r="S12" s="12"/>
       <c r="T12" s="12"/>
-      <c r="U12" s="12"/>
-      <c r="V12" s="28">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="W12">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="U12" s="28"/>
+      <c r="V12">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A13" s="11"/>
       <c r="B13" s="11"/>
       <c r="C13" s="12"/>
@@ -12304,117 +12317,101 @@
       <c r="G13" s="12"/>
       <c r="H13" s="12"/>
       <c r="I13" s="12"/>
-      <c r="J13" s="28">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="K13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="L13" s="41" t="s">
-        <v>29</v>
-      </c>
+      <c r="J13">
+        <f>SUM(C13:F13,G13,H13,I13)/40</f>
+        <v>0</v>
+      </c>
+      <c r="K13" s="41"/>
+      <c r="L13" s="11"/>
       <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
+      <c r="N13" s="12"/>
       <c r="O13" s="12"/>
       <c r="P13" s="12"/>
-      <c r="Q13" s="12"/>
-      <c r="R13" s="28">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
+      <c r="Q13" s="28"/>
+      <c r="R13" s="12"/>
       <c r="S13" s="12"/>
       <c r="T13" s="12"/>
-      <c r="U13" s="12"/>
-      <c r="V13" s="28">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="W13">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
+      <c r="U13" s="28"/>
+      <c r="V13">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A14" s="13"/>
       <c r="B14" s="10"/>
       <c r="C14" s="14">
-        <f t="shared" ref="C14:J14" si="5">SUM(C8:C13)</f>
-        <v>0</v>
+        <f t="shared" ref="C14:I14" si="1">SUM(C8:C13)</f>
+        <v>754</v>
       </c>
       <c r="D14" s="14">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>164</v>
       </c>
       <c r="E14" s="14">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>164</v>
       </c>
       <c r="F14" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="G14" s="14">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>363</v>
       </c>
       <c r="H14" s="14">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f t="shared" si="1"/>
+        <v>236</v>
       </c>
       <c r="I14" s="14">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="J14" s="14">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="K14" s="35">
+        <f t="shared" si="1"/>
+        <v>369</v>
+      </c>
+      <c r="J14" s="35">
         <f>C14+D14+E14+F14+G14+H14+I14</f>
-        <v>0</v>
-      </c>
-      <c r="M14" s="13"/>
-      <c r="N14" s="10"/>
+        <v>2050</v>
+      </c>
+      <c r="L14" s="13"/>
+      <c r="M14" s="10"/>
+      <c r="N14" s="14">
+        <f t="shared" ref="N14:U14" si="2">SUM(N8:N13)</f>
+        <v>0</v>
+      </c>
       <c r="O14" s="14">
-        <f t="shared" ref="O14:V14" si="6">SUM(O8:O13)</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="P14" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="Q14" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="R14" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="S14" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="T14" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="U14" s="14">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="V14" s="14">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="W14" s="35" t="e">
-        <f>O14+P14+Q14+#REF!+S14+T14+U14</f>
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="V14" s="35" t="e">
+        <f>N14+O14+P14+#REF!+R14+S14+T14</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A15" s="13"/>
       <c r="B15" s="10" t="s">
         <v>22</v>
@@ -12422,199 +12419,196 @@
       <c r="C15" s="13"/>
       <c r="D15" s="13">
         <f>D14/20</f>
-        <v>0</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="E15" s="13">
-        <f t="shared" ref="E15:I15" si="7">E14/20</f>
-        <v>0</v>
+        <f t="shared" ref="E15:I15" si="3">E14/20</f>
+        <v>8.1999999999999993</v>
       </c>
       <c r="F15" s="13">
-        <f t="shared" si="7"/>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="G15" s="13">
-        <f t="shared" si="7"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>18.149999999999999</v>
       </c>
       <c r="H15" s="13">
-        <f t="shared" si="7"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>11.8</v>
       </c>
       <c r="I15" s="13">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="J15" s="13"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="10" t="s">
+        <f t="shared" si="3"/>
+        <v>18.45</v>
+      </c>
+      <c r="L15" s="13"/>
+      <c r="M15" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="O15" s="13"/>
+      <c r="N15" s="13"/>
+      <c r="O15" s="13">
+        <f>O14/20</f>
+        <v>0</v>
+      </c>
       <c r="P15" s="13">
-        <f>P14/20</f>
-        <v>0</v>
-      </c>
-      <c r="Q15" s="13">
-        <f t="shared" ref="Q15" si="8">Q14/20</f>
-        <v>0</v>
-      </c>
-      <c r="R15" s="13"/>
+        <f t="shared" ref="P15" si="4">P14/20</f>
+        <v>0</v>
+      </c>
+      <c r="Q15" s="13"/>
+      <c r="R15" s="13">
+        <f t="shared" ref="R15:T15" si="5">R14/20</f>
+        <v>0</v>
+      </c>
       <c r="S15" s="13">
-        <f t="shared" ref="S15:U15" si="9">S14/20</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="T15" s="13">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="U15" s="13">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="V15" s="13"/>
-    </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="U15" s="13"/>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A16" s="13"/>
       <c r="B16" s="10" t="s">
         <v>21</v>
       </c>
       <c r="C16" s="36">
         <f>C15+C14</f>
-        <v>0</v>
+        <v>754</v>
       </c>
       <c r="D16" s="36">
-        <f t="shared" ref="D16:I16" si="10">D15+D14</f>
-        <v>0</v>
+        <f t="shared" ref="D16:I16" si="6">D15+D14</f>
+        <v>172.2</v>
       </c>
       <c r="E16" s="36">
-        <f t="shared" si="10"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>172.2</v>
       </c>
       <c r="F16" s="36">
-        <f t="shared" si="10"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="G16" s="36">
-        <f t="shared" si="10"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>381.15</v>
       </c>
       <c r="H16" s="36">
-        <f t="shared" si="10"/>
-        <v>0</v>
+        <f t="shared" si="6"/>
+        <v>247.8</v>
       </c>
       <c r="I16" s="36">
-        <f t="shared" si="10"/>
-        <v>0</v>
-      </c>
-      <c r="J16" s="36"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="10" t="s">
+        <f t="shared" si="6"/>
+        <v>387.45</v>
+      </c>
+      <c r="L16" s="13"/>
+      <c r="M16" s="10" t="s">
         <v>21</v>
       </c>
+      <c r="N16" s="36">
+        <f>N15+N14</f>
+        <v>0</v>
+      </c>
       <c r="O16" s="36">
-        <f>O15+O14</f>
+        <f t="shared" ref="O16:P16" si="7">O15+O14</f>
         <v>0</v>
       </c>
       <c r="P16" s="36">
-        <f t="shared" ref="P16:Q16" si="11">P15+P14</f>
-        <v>0</v>
-      </c>
-      <c r="Q16" s="36">
-        <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="R16" s="36"/>
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="Q16" s="36"/>
+      <c r="R16" s="36">
+        <f t="shared" ref="R16:T16" si="8">R15+R14</f>
+        <v>0</v>
+      </c>
       <c r="S16" s="36">
-        <f t="shared" ref="S16:U16" si="12">S15+S14</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
       <c r="T16" s="36">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="U16" s="36">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="V16" s="36"/>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+      <c r="U16" s="36"/>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A17" s="13"/>
       <c r="B17" s="39" t="s">
         <v>23</v>
       </c>
       <c r="C17" s="36">
         <f>C14/40</f>
-        <v>0</v>
+        <v>18.850000000000001</v>
       </c>
       <c r="D17" s="36">
-        <f t="shared" ref="D17:I17" si="13">D14/40</f>
-        <v>0</v>
+        <f t="shared" ref="D17:I17" si="9">D14/40</f>
+        <v>4.0999999999999996</v>
       </c>
       <c r="E17" s="36">
-        <f t="shared" si="13"/>
-        <v>0</v>
+        <f t="shared" si="9"/>
+        <v>4.0999999999999996</v>
       </c>
       <c r="F17" s="36">
-        <f t="shared" si="13"/>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="G17" s="36">
-        <f t="shared" si="13"/>
-        <v>0</v>
+        <f t="shared" si="9"/>
+        <v>9.0749999999999993</v>
       </c>
       <c r="H17" s="36">
-        <f t="shared" si="13"/>
-        <v>0</v>
+        <f t="shared" si="9"/>
+        <v>5.9</v>
       </c>
       <c r="I17" s="36">
-        <f t="shared" si="13"/>
-        <v>0</v>
-      </c>
-      <c r="J17" s="36"/>
-      <c r="K17" s="35">
+        <f t="shared" si="9"/>
+        <v>9.2249999999999996</v>
+      </c>
+      <c r="J17" s="35">
         <f>SUM(C17:I17)</f>
-        <v>0</v>
-      </c>
-      <c r="M17" s="13"/>
-      <c r="N17" s="39" t="s">
+        <v>51.25</v>
+      </c>
+      <c r="L17" s="13"/>
+      <c r="M17" s="39" t="s">
         <v>23</v>
       </c>
+      <c r="N17" s="36">
+        <f>N14/40</f>
+        <v>0</v>
+      </c>
       <c r="O17" s="36">
-        <f>O14/40</f>
+        <f t="shared" ref="O17:P17" si="10">O14/40</f>
         <v>0</v>
       </c>
       <c r="P17" s="36">
-        <f t="shared" ref="P17:Q17" si="14">P14/40</f>
-        <v>0</v>
-      </c>
-      <c r="Q17" s="36">
-        <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="R17" s="36"/>
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="Q17" s="36"/>
+      <c r="R17" s="36">
+        <f t="shared" ref="R17:T17" si="11">R14/40</f>
+        <v>0</v>
+      </c>
       <c r="S17" s="36">
-        <f t="shared" ref="S17:U17" si="15">S14/40</f>
+        <f t="shared" si="11"/>
         <v>0</v>
       </c>
       <c r="T17" s="36">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="U17" s="36">
-        <f t="shared" si="15"/>
-        <v>0</v>
-      </c>
-      <c r="V17" s="36"/>
-      <c r="W17" s="35">
-        <f>SUM(O17:U17)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
+        <f t="shared" si="11"/>
+        <v>0</v>
+      </c>
+      <c r="U17" s="36"/>
+      <c r="V17" s="35">
+        <f>SUM(N17:T17)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
       <c r="C18" s="32"/>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="26"/>
@@ -12624,16 +12618,15 @@
       <c r="G19" s="26"/>
       <c r="H19" s="26"/>
       <c r="I19" s="26"/>
-      <c r="J19" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B2:J5"/>
+    <mergeCell ref="B2:I5"/>
     <mergeCell ref="D6:F6"/>
-    <mergeCell ref="G6:J6"/>
-    <mergeCell ref="N2:V5"/>
-    <mergeCell ref="P6:R6"/>
-    <mergeCell ref="S6:V6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="M2:U5"/>
+    <mergeCell ref="O6:Q6"/>
+    <mergeCell ref="R6:U6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12686,7 +12679,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -12698,7 +12691,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -12974,7 +12967,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="43" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="29"/>
       <c r="D10" s="29"/>
@@ -13018,7 +13011,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -13484,7 +13477,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -13496,7 +13489,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -13778,7 +13771,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -13825,7 +13818,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -14308,7 +14301,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -14320,7 +14313,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -14602,7 +14595,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -14649,7 +14642,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -15107,7 +15100,7 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
@@ -15119,7 +15112,7 @@
       <c r="O1" s="1"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
@@ -15130,7 +15123,7 @@
     <row r="2" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -15142,7 +15135,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -15441,7 +15434,7 @@
     <row r="10" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -15495,7 +15488,7 @@
     <row r="11" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -15981,7 +15974,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -15993,7 +15986,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -16269,7 +16262,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -16313,7 +16306,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -16779,7 +16772,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -16791,7 +16784,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -17067,7 +17060,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -17111,7 +17104,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -17580,7 +17573,7 @@
     <row r="2" spans="1:25" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -17592,7 +17585,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -17891,7 +17884,7 @@
     <row r="10" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -17943,7 +17936,7 @@
     <row r="11" spans="1:25" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -18430,7 +18423,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -18442,7 +18435,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -18724,7 +18717,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -18771,7 +18764,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -19245,7 +19238,7 @@
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -19258,7 +19251,7 @@
       <c r="K2" s="63"/>
       <c r="N2" s="1"/>
       <c r="O2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P2" s="62"/>
       <c r="Q2" s="62"/>
@@ -19637,7 +19630,7 @@
         <v>46175</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>60</v>
@@ -19722,7 +19715,7 @@
         <v>46175</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>276</v>
@@ -19882,7 +19875,7 @@
         <v>46175</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="12">
@@ -20330,7 +20323,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -20342,7 +20335,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -20618,7 +20611,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -20662,7 +20655,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -21128,7 +21121,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -21140,7 +21133,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -21416,7 +21409,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -21460,7 +21453,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -21927,7 +21920,7 @@
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -21939,7 +21932,7 @@
       <c r="J2" s="63"/>
       <c r="M2" s="1"/>
       <c r="N2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
@@ -22215,7 +22208,7 @@
     <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="12"/>
@@ -22259,7 +22252,7 @@
     <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="12"/>
@@ -22727,7 +22720,7 @@
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -22740,7 +22733,7 @@
       <c r="K2" s="63"/>
       <c r="N2" s="1"/>
       <c r="O2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P2" s="62"/>
       <c r="Q2" s="62"/>
@@ -23102,7 +23095,7 @@
         <v>46176</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>100</v>
@@ -23189,7 +23182,7 @@
         <v>46176</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>612</v>
@@ -23361,7 +23354,7 @@
         <v>46176</v>
       </c>
       <c r="O13" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="P13" s="12"/>
       <c r="Q13" s="12">
@@ -23771,7 +23764,7 @@
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -23784,7 +23777,7 @@
       <c r="K2" s="63"/>
       <c r="N2" s="1"/>
       <c r="O2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P2" s="62"/>
       <c r="Q2" s="62"/>
@@ -24146,7 +24139,7 @@
         <v>46177</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>262</v>
@@ -24233,7 +24226,7 @@
         <v>46177</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>182</v>
@@ -24406,7 +24399,7 @@
     <row r="13" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A13" s="11"/>
       <c r="B13" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" s="12"/>
       <c r="D13" s="12">
@@ -24838,7 +24831,7 @@
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -24851,7 +24844,7 @@
       <c r="K2" s="63"/>
       <c r="N2" s="1"/>
       <c r="O2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P2" s="62"/>
       <c r="Q2" s="62"/>
@@ -25608,7 +25601,7 @@
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -25621,7 +25614,7 @@
       <c r="K2" s="63"/>
       <c r="N2" s="1"/>
       <c r="O2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P2" s="62"/>
       <c r="Q2" s="62"/>
@@ -25955,7 +25948,7 @@
     <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>200</v>
@@ -26033,7 +26026,7 @@
     <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11" s="10"/>
       <c r="B11" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>280</v>
@@ -26481,7 +26474,7 @@
     <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -26494,7 +26487,7 @@
       <c r="K2" s="63"/>
       <c r="N2" s="1"/>
       <c r="O2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="P2" s="62"/>
       <c r="Q2" s="62"/>
@@ -26837,7 +26830,7 @@
     <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>40</v>
@@ -26911,7 +26904,7 @@
     <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>242</v>
@@ -27456,7 +27449,7 @@
     <row r="2" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
@@ -27467,7 +27460,7 @@
       <c r="I2" s="63"/>
       <c r="L2" s="1"/>
       <c r="M2" s="61" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N2" s="62"/>
       <c r="O2" s="62"/>
@@ -27786,7 +27779,7 @@
         <v>46181</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="12">
         <v>40</v>
@@ -27890,7 +27883,7 @@
     <row r="12" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A12" s="11"/>
       <c r="B12" s="11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" s="12">
         <v>254</v>

</xml_diff>

<commit_message>
morning update after booking complete
</commit_message>
<xml_diff>
--- a/july 2026/Daily Reports/Final Execution SKU wise  july.xlsx
+++ b/july 2026/Daily Reports/Final Execution SKU wise  july.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\786\Desktop\Elite-Git\july 2026\Daily Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54507373-020E-4835-B38F-BBF9C46AA3B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA09A7B3-4048-45C7-8033-884E8473E2C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="887" activeTab="21" xr2:uid="{6D56E189-8B51-44FA-B14F-5373D35B2784}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1383" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1384" uniqueCount="44">
   <si>
     <t>Gate Pass</t>
   </si>
@@ -185,6 +185,9 @@
   </si>
   <si>
     <t>120lem</t>
+  </si>
+  <si>
+    <t>No EXC</t>
   </si>
 </sst>
 </file>
@@ -667,7 +670,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
@@ -849,11 +852,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -11861,7 +11861,7 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C45487-B908-4B5C-9BA4-6B5B2A14CAC7}">
-  <dimension ref="A1:W19"/>
+  <dimension ref="A1:V19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3.90625" bestFit="1" customWidth="1"/>
@@ -11877,10 +11877,9 @@
     <col min="14" max="14" width="4" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="5" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="4.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -11899,9 +11898,8 @@
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
-      <c r="U1" s="1"/>
-    </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="61" t="s">
         <v>34</v>
@@ -11923,10 +11921,9 @@
       <c r="Q2" s="62"/>
       <c r="R2" s="62"/>
       <c r="S2" s="62"/>
-      <c r="T2" s="62"/>
-      <c r="U2" s="63"/>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="T2" s="63"/>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="64"/>
       <c r="C3" s="65"/>
@@ -11944,10 +11941,9 @@
       <c r="Q3" s="65"/>
       <c r="R3" s="65"/>
       <c r="S3" s="65"/>
-      <c r="T3" s="65"/>
-      <c r="U3" s="66"/>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="T3" s="66"/>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="B4" s="64"/>
       <c r="C4" s="65"/>
@@ -11965,10 +11961,9 @@
       <c r="Q4" s="65"/>
       <c r="R4" s="65"/>
       <c r="S4" s="65"/>
-      <c r="T4" s="65"/>
-      <c r="U4" s="66"/>
-    </row>
-    <row r="5" spans="1:23" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="T4" s="66"/>
+    </row>
+    <row r="5" spans="1:22" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="1"/>
       <c r="B5" s="67"/>
       <c r="C5" s="68"/>
@@ -11986,10 +11981,9 @@
       <c r="Q5" s="68"/>
       <c r="R5" s="68"/>
       <c r="S5" s="68"/>
-      <c r="T5" s="68"/>
-      <c r="U5" s="69"/>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="T5" s="69"/>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
       <c r="B6" s="2"/>
       <c r="C6" s="3" t="s">
@@ -12019,10 +12013,9 @@
         <v>3</v>
       </c>
       <c r="S6" s="71"/>
-      <c r="T6" s="71"/>
-      <c r="U6" s="72"/>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="T6" s="72"/>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>4</v>
       </c>
@@ -12081,19 +12074,16 @@
         <v>7</v>
       </c>
       <c r="T7" s="45" t="s">
-        <v>12</v>
-      </c>
-      <c r="U7" s="45" t="s">
         <v>8</v>
       </c>
+      <c r="U7" s="12" t="s">
+        <v>27</v>
+      </c>
       <c r="V7" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="W7" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A8" s="27"/>
       <c r="B8" s="10" t="s">
         <v>17</v>
@@ -12118,17 +12108,16 @@
       <c r="N8" s="28"/>
       <c r="O8" s="12"/>
       <c r="P8" s="12"/>
-      <c r="Q8" s="75"/>
-      <c r="R8" s="75"/>
-      <c r="S8" s="75"/>
-      <c r="T8" s="75"/>
-      <c r="U8" s="75"/>
-      <c r="V8">
-        <f t="shared" ref="V8:V13" si="1">SUM(N8:P8,R8,S8,T8)/40</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="Q8" s="12"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="12"/>
+      <c r="T8" s="12"/>
+      <c r="U8">
+        <f t="shared" ref="U8:U9" si="1">SUM(N8:T8)/40</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A9" s="27"/>
       <c r="B9" s="10" t="s">
         <v>14</v>
@@ -12166,20 +12155,22 @@
         <f>B9</f>
         <v>Salman</v>
       </c>
-      <c r="N9" s="28"/>
-      <c r="O9" s="12"/>
-      <c r="P9" s="12"/>
-      <c r="Q9" s="75"/>
-      <c r="R9" s="75"/>
-      <c r="S9" s="75"/>
-      <c r="T9" s="75"/>
-      <c r="U9" s="75"/>
-      <c r="V9">
+      <c r="N9" s="29"/>
+      <c r="O9" s="29"/>
+      <c r="P9" s="29"/>
+      <c r="Q9" s="29"/>
+      <c r="R9" s="29"/>
+      <c r="S9" s="29"/>
+      <c r="T9" s="29"/>
+      <c r="U9">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="V9" s="42" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A10" s="27"/>
       <c r="B10" s="10" t="s">
         <v>37</v>
@@ -12217,20 +12208,36 @@
         <f>B10</f>
         <v>Zesahn</v>
       </c>
-      <c r="N10" s="28"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="12"/>
-      <c r="Q10" s="75"/>
-      <c r="R10" s="75"/>
-      <c r="S10" s="75"/>
-      <c r="T10" s="75"/>
-      <c r="U10" s="75"/>
-      <c r="V10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="N10" s="28">
+        <v>202</v>
+      </c>
+      <c r="O10" s="12">
+        <v>66</v>
+      </c>
+      <c r="P10" s="12">
+        <v>66</v>
+      </c>
+      <c r="Q10" s="12">
+        <v>0</v>
+      </c>
+      <c r="R10" s="12">
+        <v>126</v>
+      </c>
+      <c r="S10" s="12">
+        <v>126</v>
+      </c>
+      <c r="T10" s="12">
+        <v>212</v>
+      </c>
+      <c r="U10">
+        <f>SUM(N10:T10)/40</f>
+        <v>19.95</v>
+      </c>
+      <c r="V10" s="44">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A11" s="11"/>
       <c r="B11" s="11" t="s">
         <v>31</v>
@@ -12268,55 +12275,100 @@
         <f>B11</f>
         <v>Umair</v>
       </c>
-      <c r="N11" s="28"/>
-      <c r="O11" s="12"/>
-      <c r="P11" s="12"/>
-      <c r="Q11" s="75"/>
-      <c r="R11" s="75"/>
-      <c r="S11" s="75"/>
-      <c r="T11" s="75"/>
-      <c r="U11" s="75"/>
-      <c r="V11">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="N11" s="28">
+        <v>420</v>
+      </c>
+      <c r="O11" s="12">
+        <v>80</v>
+      </c>
+      <c r="P11" s="12">
+        <v>80</v>
+      </c>
+      <c r="Q11" s="12">
+        <v>0</v>
+      </c>
+      <c r="R11" s="12">
+        <v>120</v>
+      </c>
+      <c r="S11" s="12">
+        <v>40</v>
+      </c>
+      <c r="T11" s="12">
+        <v>40</v>
+      </c>
+      <c r="U11">
+        <f>SUM(N11:T11)/40</f>
+        <v>19.5</v>
+      </c>
+      <c r="V11" s="44">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A12" s="11"/>
       <c r="B12" s="11" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
+      <c r="D12" s="12">
+        <v>1189</v>
+      </c>
+      <c r="E12" s="12">
+        <v>1395</v>
+      </c>
       <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
+      <c r="G12" s="12">
+        <v>2398</v>
+      </c>
+      <c r="H12" s="12">
+        <v>2397</v>
+      </c>
+      <c r="I12" s="12">
+        <v>4800</v>
+      </c>
       <c r="J12">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K12" s="41"/>
+        <v>304.47500000000002</v>
+      </c>
+      <c r="K12" s="41">
+        <v>1</v>
+      </c>
       <c r="L12" s="11"/>
-      <c r="M12" s="10" t="str">
-        <f>B12</f>
-        <v>Mubeen</v>
+      <c r="M12" s="10" t="s">
+        <v>38</v>
       </c>
       <c r="N12" s="28"/>
-      <c r="O12" s="12"/>
-      <c r="P12" s="12"/>
-      <c r="Q12" s="75"/>
-      <c r="R12" s="75"/>
-      <c r="S12" s="75"/>
-      <c r="T12" s="75"/>
-      <c r="U12" s="75"/>
-      <c r="V12">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="O12" s="12">
+        <f>1189+40</f>
+        <v>1229</v>
+      </c>
+      <c r="P12" s="12">
+        <f>1395+40</f>
+        <v>1435</v>
+      </c>
+      <c r="Q12" s="12">
+        <v>0</v>
+      </c>
+      <c r="R12" s="12">
+        <f>2398+40</f>
+        <v>2438</v>
+      </c>
+      <c r="S12" s="12">
+        <v>2397</v>
+      </c>
+      <c r="T12" s="12">
+        <f>4800+40</f>
+        <v>4840</v>
+      </c>
+      <c r="U12">
+        <f>SUM(N12:T12)/40</f>
+        <v>308.47500000000002</v>
+      </c>
+      <c r="V12" s="44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A13" s="11"/>
       <c r="B13" s="11"/>
       <c r="C13" s="12"/>
@@ -12336,17 +12388,16 @@
       <c r="N13" s="12"/>
       <c r="O13" s="12"/>
       <c r="P13" s="12"/>
-      <c r="Q13" s="75"/>
-      <c r="R13" s="75"/>
-      <c r="S13" s="75"/>
-      <c r="T13" s="75"/>
-      <c r="U13" s="75"/>
-      <c r="V13">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.35">
+      <c r="Q13" s="12"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="12"/>
+      <c r="T13" s="12"/>
+      <c r="U13">
+        <f>SUM(N13:T13)/40</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A14" s="13"/>
       <c r="B14" s="10"/>
       <c r="C14" s="14">
@@ -12355,11 +12406,11 @@
       </c>
       <c r="D14" s="14">
         <f t="shared" si="2"/>
-        <v>164</v>
+        <v>1353</v>
       </c>
       <c r="E14" s="14">
         <f t="shared" si="2"/>
-        <v>164</v>
+        <v>1559</v>
       </c>
       <c r="F14" s="14">
         <f t="shared" si="2"/>
@@ -12367,33 +12418,33 @@
       </c>
       <c r="G14" s="14">
         <f t="shared" si="2"/>
-        <v>363</v>
+        <v>2761</v>
       </c>
       <c r="H14" s="14">
         <f t="shared" si="2"/>
-        <v>236</v>
+        <v>2633</v>
       </c>
       <c r="I14" s="14">
         <f t="shared" si="2"/>
-        <v>369</v>
+        <v>5169</v>
       </c>
       <c r="J14" s="35">
         <f>C14+D14+E14+F14+G14+H14+I14</f>
-        <v>2050</v>
+        <v>14229</v>
       </c>
       <c r="L14" s="13"/>
       <c r="M14" s="10"/>
       <c r="N14" s="14">
-        <f t="shared" ref="N14:U14" si="3">SUM(N8:N13)</f>
-        <v>0</v>
+        <f t="shared" ref="N14:T14" si="3">SUM(N8:N13)</f>
+        <v>622</v>
       </c>
       <c r="O14" s="14">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1375</v>
       </c>
       <c r="P14" s="14">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1581</v>
       </c>
       <c r="Q14" s="14">
         <f t="shared" si="3"/>
@@ -12401,26 +12452,22 @@
       </c>
       <c r="R14" s="14">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2684</v>
       </c>
       <c r="S14" s="14">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2563</v>
       </c>
       <c r="T14" s="14">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="U14" s="14">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="V14" s="35" t="e">
-        <f>N14+O14+P14+#REF!+R14+S14+T14</f>
+        <v>5092</v>
+      </c>
+      <c r="U14" s="35" t="e">
+        <f>N14+O14+P14+#REF!+R14+S14+#REF!</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A15" s="13"/>
       <c r="B15" s="10" t="s">
         <v>22</v>
@@ -12428,11 +12475,11 @@
       <c r="C15" s="13"/>
       <c r="D15" s="13">
         <f>D14/20</f>
-        <v>8.1999999999999993</v>
+        <v>67.650000000000006</v>
       </c>
       <c r="E15" s="13">
         <f t="shared" ref="E15:I15" si="4">E14/20</f>
-        <v>8.1999999999999993</v>
+        <v>77.95</v>
       </c>
       <c r="F15" s="13">
         <f t="shared" si="4"/>
@@ -12440,15 +12487,15 @@
       </c>
       <c r="G15" s="13">
         <f t="shared" si="4"/>
-        <v>18.149999999999999</v>
+        <v>138.05000000000001</v>
       </c>
       <c r="H15" s="13">
         <f t="shared" si="4"/>
-        <v>11.8</v>
+        <v>131.65</v>
       </c>
       <c r="I15" s="13">
         <f t="shared" si="4"/>
-        <v>18.45</v>
+        <v>258.45</v>
       </c>
       <c r="L15" s="13"/>
       <c r="M15" s="10" t="s">
@@ -12457,28 +12504,24 @@
       <c r="N15" s="13"/>
       <c r="O15" s="13">
         <f>O14/20</f>
-        <v>0</v>
+        <v>68.75</v>
       </c>
       <c r="P15" s="13">
         <f t="shared" ref="P15" si="5">P14/20</f>
-        <v>0</v>
+        <v>79.05</v>
       </c>
       <c r="Q15" s="13"/>
       <c r="R15" s="13">
-        <f t="shared" ref="R15:T15" si="6">R14/20</f>
-        <v>0</v>
+        <f t="shared" ref="R15:S15" si="6">R14/20</f>
+        <v>134.19999999999999</v>
       </c>
       <c r="S15" s="13">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="T15" s="13">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="U15" s="13"/>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.35">
+        <v>128.15</v>
+      </c>
+      <c r="T15" s="13"/>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A16" s="13"/>
       <c r="B16" s="10" t="s">
         <v>21</v>
@@ -12489,11 +12532,11 @@
       </c>
       <c r="D16" s="36">
         <f t="shared" ref="D16:I16" si="7">D15+D14</f>
-        <v>172.2</v>
+        <v>1420.65</v>
       </c>
       <c r="E16" s="36">
         <f t="shared" si="7"/>
-        <v>172.2</v>
+        <v>1636.95</v>
       </c>
       <c r="F16" s="36">
         <f t="shared" si="7"/>
@@ -12501,15 +12544,15 @@
       </c>
       <c r="G16" s="36">
         <f t="shared" si="7"/>
-        <v>381.15</v>
+        <v>2899.05</v>
       </c>
       <c r="H16" s="36">
         <f t="shared" si="7"/>
-        <v>247.8</v>
+        <v>2764.65</v>
       </c>
       <c r="I16" s="36">
         <f t="shared" si="7"/>
-        <v>387.45</v>
+        <v>5427.45</v>
       </c>
       <c r="L16" s="13"/>
       <c r="M16" s="10" t="s">
@@ -12517,32 +12560,28 @@
       </c>
       <c r="N16" s="36">
         <f>N15+N14</f>
-        <v>0</v>
+        <v>622</v>
       </c>
       <c r="O16" s="36">
         <f t="shared" ref="O16:P16" si="8">O15+O14</f>
-        <v>0</v>
+        <v>1443.75</v>
       </c>
       <c r="P16" s="36">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>1660.05</v>
       </c>
       <c r="Q16" s="36"/>
       <c r="R16" s="36">
-        <f t="shared" ref="R16:T16" si="9">R15+R14</f>
-        <v>0</v>
+        <f t="shared" ref="R16:S16" si="9">R15+R14</f>
+        <v>2818.2</v>
       </c>
       <c r="S16" s="36">
         <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="T16" s="36">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="U16" s="36"/>
-    </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+        <v>2691.15</v>
+      </c>
+      <c r="T16" s="36"/>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A17" s="13"/>
       <c r="B17" s="39" t="s">
         <v>23</v>
@@ -12553,11 +12592,11 @@
       </c>
       <c r="D17" s="36">
         <f t="shared" ref="D17:I17" si="10">D14/40</f>
-        <v>4.0999999999999996</v>
+        <v>33.825000000000003</v>
       </c>
       <c r="E17" s="36">
         <f t="shared" si="10"/>
-        <v>4.0999999999999996</v>
+        <v>38.975000000000001</v>
       </c>
       <c r="F17" s="36">
         <f t="shared" si="10"/>
@@ -12565,19 +12604,19 @@
       </c>
       <c r="G17" s="36">
         <f t="shared" si="10"/>
-        <v>9.0749999999999993</v>
+        <v>69.025000000000006</v>
       </c>
       <c r="H17" s="36">
         <f t="shared" si="10"/>
-        <v>5.9</v>
+        <v>65.825000000000003</v>
       </c>
       <c r="I17" s="36">
         <f t="shared" si="10"/>
-        <v>9.2249999999999996</v>
+        <v>129.22499999999999</v>
       </c>
       <c r="J17" s="35">
         <f>SUM(C17:I17)</f>
-        <v>51.25</v>
+        <v>355.72500000000002</v>
       </c>
       <c r="L17" s="13"/>
       <c r="M17" s="39" t="s">
@@ -12585,39 +12624,35 @@
       </c>
       <c r="N17" s="36">
         <f>N14/40</f>
-        <v>0</v>
+        <v>15.55</v>
       </c>
       <c r="O17" s="36">
         <f t="shared" ref="O17:P17" si="11">O14/40</f>
-        <v>0</v>
+        <v>34.375</v>
       </c>
       <c r="P17" s="36">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>39.524999999999999</v>
       </c>
       <c r="Q17" s="36"/>
       <c r="R17" s="36">
-        <f t="shared" ref="R17:T17" si="12">R14/40</f>
-        <v>0</v>
+        <f t="shared" ref="R17:S17" si="12">R14/40</f>
+        <v>67.099999999999994</v>
       </c>
       <c r="S17" s="36">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="T17" s="36">
-        <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="U17" s="36"/>
-      <c r="V17" s="35">
-        <f>SUM(N17:T17)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+        <v>64.075000000000003</v>
+      </c>
+      <c r="T17" s="36"/>
+      <c r="U17" s="35">
+        <f>SUM(N17:S17)</f>
+        <v>220.625</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.35">
       <c r="C18" s="32"/>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="26"/>
@@ -12633,9 +12668,9 @@
     <mergeCell ref="B2:I5"/>
     <mergeCell ref="D6:F6"/>
     <mergeCell ref="G6:I6"/>
-    <mergeCell ref="M2:U5"/>
+    <mergeCell ref="M2:T5"/>
     <mergeCell ref="O6:Q6"/>
-    <mergeCell ref="R6:U6"/>
+    <mergeCell ref="R6:T6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13001,30 +13036,32 @@
         <v>37</v>
       </c>
       <c r="C10" s="28">
-        <v>80</v>
+        <v>244</v>
       </c>
       <c r="D10" s="12">
         <v>40</v>
       </c>
       <c r="E10" s="12">
-        <v>40</v>
-      </c>
-      <c r="F10" s="12"/>
+        <v>0</v>
+      </c>
+      <c r="F10" s="12">
+        <v>0</v>
+      </c>
       <c r="G10" s="12">
-        <v>85</v>
+        <v>105</v>
       </c>
       <c r="H10" s="12">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="I10" s="12">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="J10">
         <f>SUM(C10:F10,G10,H10,I10)/40</f>
-        <v>9.9749999999999996</v>
+        <v>12.1</v>
       </c>
       <c r="K10" s="44">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="L10" s="27"/>
       <c r="M10" s="10" t="str">
@@ -13098,23 +13135,36 @@
     <row r="12" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A12" s="11"/>
       <c r="B12" s="11" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="C12" s="28"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
+      <c r="D12" s="12">
+        <v>800</v>
+      </c>
+      <c r="E12" s="12">
+        <v>1280</v>
+      </c>
       <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-      <c r="I12" s="12"/>
+      <c r="G12" s="12">
+        <v>1040</v>
+      </c>
+      <c r="H12" s="12">
+        <v>1280</v>
+      </c>
+      <c r="I12" s="12">
+        <v>1520</v>
+      </c>
       <c r="J12">
         <f>SUM(C12:F12,G12,H12,I12)/40</f>
-        <v>0</v>
+        <v>148</v>
+      </c>
+      <c r="K12" s="75">
+        <v>7</v>
       </c>
       <c r="L12" s="11"/>
       <c r="M12" s="10" t="str">
         <f>B12</f>
-        <v>Mubeen</v>
+        <v xml:space="preserve">Shakoor </v>
       </c>
       <c r="N12" s="28"/>
       <c r="O12" s="12"/>
@@ -13159,15 +13209,15 @@
       <c r="B14" s="10"/>
       <c r="C14" s="14">
         <f t="shared" ref="C14:I14" si="1">SUM(C8:C13)</f>
-        <v>477</v>
+        <v>641</v>
       </c>
       <c r="D14" s="14">
         <f t="shared" si="1"/>
-        <v>124</v>
+        <v>924</v>
       </c>
       <c r="E14" s="14">
         <f t="shared" si="1"/>
-        <v>129</v>
+        <v>1369</v>
       </c>
       <c r="F14" s="14">
         <f t="shared" si="1"/>
@@ -13175,19 +13225,19 @@
       </c>
       <c r="G14" s="14">
         <f t="shared" si="1"/>
-        <v>233</v>
+        <v>1293</v>
       </c>
       <c r="H14" s="14">
         <f t="shared" si="1"/>
-        <v>198</v>
+        <v>1448</v>
       </c>
       <c r="I14" s="14">
         <f t="shared" si="1"/>
-        <v>272</v>
+        <v>1763</v>
       </c>
       <c r="J14" s="35">
         <f>C14+D14+E14+F14+G14+H14+I14</f>
-        <v>1433</v>
+        <v>7438</v>
       </c>
       <c r="L14" s="13"/>
       <c r="M14" s="10"/>
@@ -13236,11 +13286,11 @@
       <c r="C15" s="13"/>
       <c r="D15" s="13">
         <f>D14/20</f>
-        <v>6.2</v>
+        <v>46.2</v>
       </c>
       <c r="E15" s="13">
         <f t="shared" ref="E15:I15" si="3">E14/20</f>
-        <v>6.45</v>
+        <v>68.45</v>
       </c>
       <c r="F15" s="13">
         <f t="shared" si="3"/>
@@ -13248,15 +13298,15 @@
       </c>
       <c r="G15" s="13">
         <f t="shared" si="3"/>
-        <v>11.65</v>
+        <v>64.650000000000006</v>
       </c>
       <c r="H15" s="13">
         <f t="shared" si="3"/>
-        <v>9.9</v>
+        <v>72.400000000000006</v>
       </c>
       <c r="I15" s="13">
         <f t="shared" si="3"/>
-        <v>13.6</v>
+        <v>88.15</v>
       </c>
       <c r="L15" s="13"/>
       <c r="M15" s="10" t="s">
@@ -13293,15 +13343,15 @@
       </c>
       <c r="C16" s="36">
         <f>C15+C14</f>
-        <v>477</v>
+        <v>641</v>
       </c>
       <c r="D16" s="36">
         <f t="shared" ref="D16:I16" si="6">D15+D14</f>
-        <v>130.19999999999999</v>
+        <v>970.2</v>
       </c>
       <c r="E16" s="36">
         <f t="shared" si="6"/>
-        <v>135.44999999999999</v>
+        <v>1437.45</v>
       </c>
       <c r="F16" s="36">
         <f t="shared" si="6"/>
@@ -13309,15 +13359,15 @@
       </c>
       <c r="G16" s="36">
         <f t="shared" si="6"/>
-        <v>244.65</v>
+        <v>1357.65</v>
       </c>
       <c r="H16" s="36">
         <f t="shared" si="6"/>
-        <v>207.9</v>
+        <v>1520.4</v>
       </c>
       <c r="I16" s="36">
         <f t="shared" si="6"/>
-        <v>285.60000000000002</v>
+        <v>1851.15</v>
       </c>
       <c r="L16" s="13"/>
       <c r="M16" s="10" t="s">
@@ -13357,15 +13407,15 @@
       </c>
       <c r="C17" s="36">
         <f>C14/40</f>
-        <v>11.925000000000001</v>
+        <v>16.024999999999999</v>
       </c>
       <c r="D17" s="36">
         <f t="shared" ref="D17:I17" si="9">D14/40</f>
-        <v>3.1</v>
+        <v>23.1</v>
       </c>
       <c r="E17" s="36">
         <f t="shared" si="9"/>
-        <v>3.2250000000000001</v>
+        <v>34.225000000000001</v>
       </c>
       <c r="F17" s="36">
         <f t="shared" si="9"/>
@@ -13373,19 +13423,19 @@
       </c>
       <c r="G17" s="36">
         <f t="shared" si="9"/>
-        <v>5.8250000000000002</v>
+        <v>32.325000000000003</v>
       </c>
       <c r="H17" s="36">
         <f t="shared" si="9"/>
-        <v>4.95</v>
+        <v>36.200000000000003</v>
       </c>
       <c r="I17" s="36">
         <f t="shared" si="9"/>
-        <v>6.8</v>
+        <v>44.075000000000003</v>
       </c>
       <c r="J17" s="35">
         <f>SUM(C17:I17)</f>
-        <v>35.824999999999996</v>
+        <v>185.95</v>
       </c>
       <c r="L17" s="13"/>
       <c r="M17" s="39" t="s">
@@ -13652,7 +13702,7 @@
       <c r="M7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="N7" s="76" t="s">
+      <c r="N7" s="37" t="s">
         <v>6</v>
       </c>
       <c r="O7" s="56" t="s">
@@ -13710,11 +13760,11 @@
       <c r="N8" s="28"/>
       <c r="O8" s="12"/>
       <c r="P8" s="12"/>
-      <c r="Q8" s="75"/>
-      <c r="R8" s="75"/>
-      <c r="S8" s="75"/>
-      <c r="T8" s="75"/>
-      <c r="U8" s="75"/>
+      <c r="Q8" s="12"/>
+      <c r="R8" s="12"/>
+      <c r="S8" s="12"/>
+      <c r="T8" s="12"/>
+      <c r="U8" s="12"/>
       <c r="V8">
         <f>SUM(N8:U8)/40</f>
         <v>0</v>
@@ -13747,11 +13797,11 @@
       <c r="N9" s="28"/>
       <c r="O9" s="12"/>
       <c r="P9" s="12"/>
-      <c r="Q9" s="75"/>
-      <c r="R9" s="75"/>
-      <c r="S9" s="75"/>
-      <c r="T9" s="75"/>
-      <c r="U9" s="75"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="12"/>
+      <c r="S9" s="12"/>
+      <c r="T9" s="12"/>
+      <c r="U9" s="12"/>
       <c r="V9">
         <f t="shared" ref="V9:V13" si="0">SUM(N9:U9)/40</f>
         <v>0</v>
@@ -13784,11 +13834,11 @@
       <c r="N10" s="28"/>
       <c r="O10" s="12"/>
       <c r="P10" s="12"/>
-      <c r="Q10" s="75"/>
-      <c r="R10" s="75"/>
-      <c r="S10" s="75"/>
-      <c r="T10" s="75"/>
-      <c r="U10" s="75"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="12"/>
+      <c r="U10" s="12"/>
       <c r="V10">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -13821,11 +13871,11 @@
       <c r="N11" s="28"/>
       <c r="O11" s="12"/>
       <c r="P11" s="12"/>
-      <c r="Q11" s="75"/>
-      <c r="R11" s="75"/>
-      <c r="S11" s="75"/>
-      <c r="T11" s="75"/>
-      <c r="U11" s="75"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="12"/>
+      <c r="S11" s="12"/>
+      <c r="T11" s="12"/>
+      <c r="U11" s="12"/>
       <c r="V11">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -13858,11 +13908,11 @@
       <c r="N12" s="28"/>
       <c r="O12" s="12"/>
       <c r="P12" s="12"/>
-      <c r="Q12" s="75"/>
-      <c r="R12" s="75"/>
-      <c r="S12" s="75"/>
-      <c r="T12" s="75"/>
-      <c r="U12" s="75"/>
+      <c r="Q12" s="12"/>
+      <c r="R12" s="12"/>
+      <c r="S12" s="12"/>
+      <c r="T12" s="12"/>
+      <c r="U12" s="12"/>
       <c r="V12">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -13883,11 +13933,11 @@
       <c r="N13" s="28"/>
       <c r="O13" s="12"/>
       <c r="P13" s="12"/>
-      <c r="Q13" s="75"/>
-      <c r="R13" s="75"/>
-      <c r="S13" s="75"/>
-      <c r="T13" s="75"/>
-      <c r="U13" s="75"/>
+      <c r="Q13" s="12"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="12"/>
+      <c r="T13" s="12"/>
+      <c r="U13" s="12"/>
       <c r="V13">
         <f t="shared" si="0"/>
         <v>0</v>

</xml_diff>